<commit_message>
fix: 补全 xlsx 缺失字段 (20列完整schema)
</commit_message>
<xml_diff>
--- a/pilot_samples.xlsx
+++ b/pilot_samples.xlsx
@@ -422,24 +422,29 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O6"/>
+  <dimension ref="A1:T6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="50" customWidth="1" min="7" max="7"/>
-    <col width="60" customWidth="1" min="8" max="8"/>
-    <col width="60" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="50" customWidth="1" min="12" max="12"/>
-    <col width="50" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="50" customWidth="1" min="11" max="11"/>
+    <col width="60" customWidth="1" min="12" max="12"/>
+    <col width="60" customWidth="1" min="13" max="13"/>
+    <col width="50" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="50" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="40" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -450,70 +455,95 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>session_id</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>turn_index</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>question</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>question_raw</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>question_type</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>sub_type</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>difficulty</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>golden_answer</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>answer_full</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>answer_keypoints</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>source_doc</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>source_page</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>relevant_chunk_ids</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>is_answerable</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>question_type</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>sub_type</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>golden_answer</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>answer_full</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>answer_keypoints</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>source_doc</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>source_page</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>relevant_chunk_ids</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>eval_notes</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>verified_by</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>verify_status</t>
         </is>
@@ -527,33 +557,53 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
+          <t>PILOT</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
           <t>安达 哮喘投保要做什么检查</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>安达 哮喘投保要做什么检查</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>generated</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>单业务细节咨询</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>健康核保</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>安达</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>easy</t>
         </is>
       </c>
-      <c r="D2" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>单业务细节咨询</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>健康核保</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>哮喘投保需提交呼吸系统问卷(NB084)；根据情况可能需医生验身(ME)或肺功能检查(PFT)（如上次病发在一个月内）；如需长期覆诊则需主诊医生报告(APS)。</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>安达对哮喘投保的核保要求包括：
 1. 填写呼吸系统问卷 NB084 (Respiratory Disease Questionnaire)
@@ -562,37 +612,42 @@
 核保方向取决于哮喘的发病年龄、病发频率、严重程度、治疗方法及吸烟习惯。</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>提交呼吸系统问卷 NB084; 如上次病发一个月内需做 ME/PFT（医生验身/肺功能检查）; 如需长期覆诊需主诊医生报告 APS</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>保司文件/安达/Chubb_常見疾病指引.pdf</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>0c047a9c_chunk_0004</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="inlineStr">
         <is>
           <t>答案仅覆盖核保要求（需要什么文件/检查），未涉及具体核保决定（标准/加费/拒保），因为核保指引表在 section_summary 类chunk中。评分时以核保要求为准即可。</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="S2" s="2" t="inlineStr">
         <is>
           <t>待人工审核</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="T2" s="2" t="inlineStr">
         <is>
           <t>draft</t>
         </is>
@@ -606,33 +661,53 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
+          <t>PILOT</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
           <t>安达高资产 免体检限额是多少</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>安达高资产 免体检限额是多少</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>generated</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>单业务细节咨询</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>产品信息</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>安达</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>easy</t>
         </is>
       </c>
-      <c r="D3" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>单业务细节咨询</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>产品信息</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>安达高资产产品(HNW)免体检限额：地区1客户18-55岁，最近两年内HNW产品总保障额≤300万美元且安达所有产品总保障额≤400万美元；地区2客户18-55岁，HNW产品≤150万美元且所有产品≤300万美元；儿童(0-17岁)总保额≤200万美元。免体检限额不适用于优良或特级优良客户。</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>安达高资产业务人寿保障产品的免体检限额规则（免體檢限額適用於以下情況）：
 1. 地区1 — 18至55岁：当前新生意申请和最近两年内的HNW产品总保障额≤300万美元，并且安达人寿最近两年内的所有产品总保障额不超过400万美元。
@@ -642,37 +717,42 @@
 HNW产品包括：世代传承保险系列(PL)、特选定期寿险系列(PTL)、凝晋人生保险计划-整付保费(AWL)、凝晋人生保险计划-定期保费(RWL)&lt;已停售&gt;、凝晋人生保险计划II-定期保费(RSL)。</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>地区1(18-55岁): HNW产品≤300万美元 + 所有产品≤400万美元; 地区2(18-55岁): HNW产品≤150万美元 + 所有产品≤300万美元; 儿童(0-17岁): 总保额≤200万美元; 免体检限额不适用于优良/特级优良客户</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>保司文件/安达/Chubb_Manual 高資產業務人壽保障產品指引 (CH) - Clean_2024Oct.pdf</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="O3" s="2" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="P3" s="2" t="inlineStr">
         <is>
           <t>52694a0a_chunk_0007</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="inlineStr">
         <is>
           <t>地区1和地区2的定义未在本chunk中出现（在文档其他部分的国家组别定义表中），评分时不应因未解释地区定义而扣分。HNW产品列表由本chunk提供，属完整信息。</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr">
+      <c r="S3" s="2" t="inlineStr">
         <is>
           <t>待人工审核</t>
         </is>
       </c>
-      <c r="O3" s="2" t="inlineStr">
+      <c r="T3" s="2" t="inlineStr">
         <is>
           <t>draft</t>
         </is>
@@ -686,33 +766,53 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
+          <t>PILOT</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
           <t>安达核保 肺结节要交什么材料 怎么看</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>安达核保 肺结节要交什么材料 怎么看</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>generated</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>单业务细节咨询</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>健康核保</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>安达</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="D4" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>单业务细节咨询</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>健康核保</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>肺结节核保需提交：(1)肿瘤问卷NB079；(2)过往肺部电脑扫描(CT)报告；(3)最近期肺部CT报告；(4)病理报告(如有)。核保方向取决于：吸烟者或非吸烟者、结节形状是否规则/病理结果、以及有无肺癌家族史。</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>安达对肺部结节(Pulmonary Nodule)的核保要求：
 **需提交材料：**
@@ -727,37 +827,42 @@
 肺结节是指直径达3厘米或以下的圆形病灶，从CT中可见是实性、半实性或磨玻璃样，有可能是早期肺癌。</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>提交肿瘤问卷 NB079; 提交过往和最近期肺部CT报告; 提交病理报告（如有）; 核保考虑吸烟史、结节形状/病理、肺癌家族史</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>保司文件/安达/Chubb_常見疾病指引.pdf</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="O4" s="2" t="inlineStr">
         <is>
           <t>13</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="P4" s="2" t="inlineStr">
         <is>
           <t>0c047a9c_chunk_0024; 0c047a9c_chunk_0025</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="R4" s="2" t="inlineStr">
         <is>
           <t>答案整合了两个chunk（核保要求+核保决定参考）。疾病背景描述chunk(0c047a9c_chunk_0023)未引用但answer_full包含了部分背景信息，如影响评分可调整。具体核保决定（标准/加费/拒保）在section_summary中，此处不涵盖。</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
+      <c r="S4" s="2" t="inlineStr">
         <is>
           <t>待人工审核</t>
         </is>
       </c>
-      <c r="O4" s="2" t="inlineStr">
+      <c r="T4" s="2" t="inlineStr">
         <is>
           <t>draft</t>
         </is>
@@ -771,33 +876,53 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
+          <t>PILOT</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
           <t>安达 私人银行客户买1000万美金寿险 要什么证明</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>安达 私人银行客户买1000万美金寿险 要什么证明</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>generated</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>单业务细节咨询</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>产品信息</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>安达</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="D5" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>单业务细节咨询</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>产品信息</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>私人银行客户(银行关系&gt;12个月)投保1000万美元(保障额在750万-3000万区间)需提交：申请书、经济状况问卷、客户背景报告及银行证明书。如银行关系&lt;12个月或资料不足，需独立收入及/或资产证明。</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>安达高资产产品财务核保指引，私人银行客户（银行关系&gt;十二个月）的财务文件要求如下：
 | 保障额（美元） | 私人银行客户（关系&gt;12个月）所需文件 |
@@ -811,37 +936,42 @@
 注意事项：如提供的证明不符合要求、不完整或不清楚，核保员保留权利要求进一步的财务要求/证明。</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>保障额750万-3000万美元: 需申请书+经济状况问卷+客户背景报告+银行证明书; 私人银行客户指银行关系&gt;12个月（参考私人银行名单）; 保障额≤200万仅需申请书披露，200万-750万需申请书+问卷+背景报告; 如证明不符合/不完整，核保员可要求进一步证明</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>保司文件/安达/Chubb_Manual 高資產業務人壽保障產品指引 (CH) - Clean_2024Oct.pdf</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="O5" s="2" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="P5" s="2" t="inlineStr">
         <is>
           <t>52694a0a_chunk_0033; 52694a0a_chunk_0034</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="R5" s="2" t="inlineStr">
         <is>
           <t>表格内容含has_table的leaf chunk。私人银行名单未在本chunk中（在文档后续章节），评分时不应要求列出具体银行。保障额区间边界值（如500万、750万、3000万）的归属可能需人工确认——表格中'5,000,001-7,500,000'和'7,500,001-30,000,000'的分界是明确的。</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="S5" s="2" t="inlineStr">
         <is>
           <t>待人工审核</t>
         </is>
       </c>
-      <c r="O5" s="2" t="inlineStr">
+      <c r="T5" s="2" t="inlineStr">
         <is>
           <t>draft</t>
         </is>
@@ -855,33 +985,53 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
+          <t>PILOT</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
           <t>安达 55岁有高血压 买500万美金寿险 体检做什么 能保吗</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>安达 55岁有高血压 买500万美金寿险 体检做什么 能保吗</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>generated</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>单业务细节咨询</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>健康核保</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>安达</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>hard</t>
         </is>
       </c>
-      <c r="D6" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>单业务细节咨询</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>健康核保</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>高血压核保要求的专项检查：医生验身(ME)、显微镜尿液分析(MU)；如病症已逾10年或客户年龄≥50岁，需加做静息心电图(Resting ECG)。核保方向取决于确诊年龄、血压控制及并发症。但「能否投保/具体加费」的核保决定表在指引摘要(section_summary)中，按标注规则无法作为出处引用，因此该部分无法给出明确答案。</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>【可回答部分——体检要求】
 高血压专项核保要求（文档2 第24页）：
@@ -895,37 +1045,42 @@
 「能否投保/加费多少」的具体核保决定表位于指引摘要（section_summary类型chunk），其内容为概括描述（"针对未确定病因的血尿，根据其程度提供人寿、危疾/早期危疾及住院保险的核保指引"格式），未对高血压给出具体判定。且按标注规则section_summary不作为标准出处。文档中仅有核保方向描述（确诊年龄、血压控制、并发症），无具体加费比例或可保性判定标准。</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>高血压专项: ME + MU + (病症≥10年或年龄≥50岁需ECG); 按保额500万验身: ME + BUP + MUC + ECG（年龄46-55, 300-500万区间）; 核保方向: 确诊年龄、血压控制及并发症; 【拒答】具体能否投保/加费比例：指引摘要(section_summary)不可作为出处，无法给出明确判定</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>保司文件/安达/Chubb_常見疾病指引.pdf; 保司文件/安达/Chubb_Manual 高資產業務人壽保障產品指引 (CH) - Clean_2024Oct.pdf</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="O6" s="2" t="inlineStr">
         <is>
           <t>24; 8</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="P6" s="2" t="inlineStr">
         <is>
           <t>0c047a9c_chunk_0067; 0c047a9c_chunk_0068; 52694a0a_chunk_0006</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="R6" s="2" t="inlineStr">
         <is>
           <t>【重点人工审核】此条设为is_answerable=false以演示拒答场景。理由：(1)「能否投保/加费比例」的核保决定表在section_summary中(0c047a9c_chunk_0069)，按规则不应引用；(2)可回答的部分（体检项目）来自两个文档三个chunk，需人工确认综合逻辑是否合理——高血压专项检查和按保额的一般验身要求有重叠(ME, ECG)，实际业务中是否取并集需核保专家确认；(3)高血压核保决定参考仅给方向（确诊年龄、血压控制、并发症），不足以做二元判定。</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="S6" s="2" t="inlineStr">
         <is>
           <t>待人工审核</t>
         </is>
       </c>
-      <c r="O6" s="2" t="inlineStr">
+      <c r="T6" s="2" t="inlineStr">
         <is>
           <t>draft</t>
         </is>

</xml_diff>